<commit_message>
Refactor domain classification to use metadata; expand README
- SDTM_Domain_Metadata.xlsx: Add Measurement column (Yes for VS, EG, MK, CV)
- COSMoS_BC_DSS_Flatten.ipynb: Replace hardcoded DOMAIN_CLASS/DOMAIN_LABEL dicts with metadata read
- Measurement_Findings.ipynb: Read Measurement flag from metadata; EG exclusion explicit
- README.md: Sharpen Why section with concrete study design example; add Key findings section covering identity patterns, collection vs ontology distinction, specimen-based diversity, DS_Code mnemonic nature, and links to analytical docs
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
+++ b/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
@@ -88,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -99,6 +99,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -697,31 +698,35 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Whether the domain is a subject-level measurement domain (VS, EG, MK, CV) (Yes/No). EG included in flag despite deferred consumer status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Brief notes on domain status or version history</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-      <c r="B26" s="2" t="n"/>
-    </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>KNOWN LIMITATIONS</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Variable-level metadata (key variables, permissible variables) is not included.</t>
         </is>
       </c>
       <c r="B28" s="2" t="n"/>
@@ -729,7 +734,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>That requires CDISC membership access to the SDTM v2.0 Excel files.</t>
+          <t>Variable-level metadata (key variables, permissible variables) is not included.</t>
         </is>
       </c>
       <c r="B29" s="2" t="n"/>
@@ -737,7 +742,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SDTM v3.0 is under review and may add or change domains.</t>
+          <t>That requires CDISC membership access to the SDTM v2.0 Excel files.</t>
         </is>
       </c>
       <c r="B30" s="2" t="n"/>
@@ -745,7 +750,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>MO (Morphology) was decommissioned in v3.4 and is not listed.</t>
+          <t>SDTM v3.0 is under review and may add or change domains.</t>
         </is>
       </c>
       <c r="B31" s="2" t="n"/>
@@ -753,10 +758,18 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>MO (Morphology) was decommissioned in v3.4 and is not listed.</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>SDTMIG section numbers are reconstructed from public sources — verify against the IG.</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -769,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -812,7 +825,12 @@
           <t>Specimen_Based</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -849,7 +867,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -882,7 +905,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -915,7 +943,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -948,7 +981,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -981,7 +1019,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1014,7 +1057,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1047,7 +1095,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1080,7 +1133,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1113,7 +1171,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1146,7 +1209,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>New in v3.4 scope</t>
         </is>
@@ -1183,7 +1251,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1216,7 +1289,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1249,7 +1327,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1282,7 +1365,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>From SDTMIG-PGx v1.0</t>
         </is>
@@ -1319,7 +1407,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1352,7 +1445,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1385,7 +1483,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1418,7 +1521,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1451,7 +1559,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1484,7 +1597,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1517,7 +1635,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1550,7 +1673,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1583,7 +1711,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1616,7 +1749,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>From SDTMIG-PGx v1.0</t>
         </is>
@@ -1653,7 +1791,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>New in v3.4</t>
         </is>
@@ -1690,7 +1833,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>New in v3.4</t>
         </is>
@@ -1727,7 +1875,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>Scope expanded in v3.4</t>
         </is>
@@ -1764,7 +1917,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1797,7 +1955,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -1830,7 +1993,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1863,7 +2031,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -1896,7 +2069,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1929,7 +2107,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>Paired with PC</t>
         </is>
@@ -1966,7 +2149,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1999,7 +2187,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>QRS instrument domain</t>
         </is>
@@ -2036,7 +2229,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -2069,7 +2267,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>QRS instrument domain</t>
         </is>
@@ -2106,7 +2309,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -2139,7 +2347,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G40" s="5" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>QRS instrument domain</t>
         </is>
@@ -2176,7 +2389,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -2209,7 +2427,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -2242,7 +2465,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -2275,7 +2503,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
         <is>
           <t>Oncology</t>
         </is>
@@ -2312,7 +2545,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
         <is>
           <t>Oncology</t>
         </is>
@@ -2349,7 +2587,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -2382,7 +2625,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -2415,7 +2663,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
         <is>
           <t>TAUG-CV</t>
         </is>
@@ -2452,7 +2705,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -2485,7 +2743,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -2518,7 +2781,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -2551,7 +2819,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -2584,7 +2857,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -2617,7 +2895,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G54" s="5" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
@@ -2650,7 +2933,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
         <is>
           <t>New in v3.4</t>
         </is>
@@ -2687,7 +2975,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G56" s="5" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
@@ -2720,7 +3013,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G57" s="5" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
         <is>
           <t>From SDTMIG-PGx v1.0</t>
         </is>

</xml_diff>

<commit_message>
Move hardcoded overrides from Extract notebook to metadata file
- SDTM_Domain_Metadata.xlsx: Add Codelist_Overrides sheet (6 rows: 4 naming
  mismatches + 2 body-system subsets) and Instrument_Domain_Rules sheet
  (3 keyword-to-domain rules). Fix Measurement header styling. Update README
  with new sheet descriptions and column documentation.
- SDTM_CT_Extract.ipynb: Read overrides and instrument rules from metadata
  instead of hardcoded dicts. Discovery logic unchanged. Output identical.
- SDTM_Test_Codes_Summary.md: Update references from hardcoded overrides
  to metadata sheets.
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
+++ b/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
@@ -9,9 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domains" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codelist_Overrides" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrument_Domain_Rules" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Domains'!$A$1:$G$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Codelist_Overrides'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Instrument_Domain_Rules'!$A$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -612,164 +616,286 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="2" t="n"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Codelist_Overrides</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CT display names that do not match Domain_Name directly (6 rows)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Keyword-to-domain mapping for non-extensible instrument codelists (3 rows)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>COLUMN DESCRIPTIONS</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Domain</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Two-letter SDTM domain abbreviation (RELREC/RELSPEC for relationship datasets)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Domain_Name</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Full domain name from SDTMIG v3.4</t>
-        </is>
-      </c>
+      <c r="B20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Observation_Class</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>SDTM observation class: Findings, Events, Interventions, Special-Purpose, Trial Design, Relationship</t>
+          <t>Two-letter SDTM domain abbreviation (RELREC/RELSPEC for relationship datasets)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>SDTMIG_Section</t>
+          <t>Domain_Name</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Section number in SDTMIG v3.4 where the domain is specified</t>
+          <t>Full domain name from SDTMIG v3.4</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Has_Test_Codes</t>
+          <t>Observation_Class</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Whether the domain uses --TESTCD/--TEST variables (Yes/No)</t>
+          <t>SDTM observation class: Findings, Events, Interventions, Special-Purpose, Trial Design, Relationship</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Specimen_Based</t>
+          <t>SDTMIG_Section</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Whether the domain is specimen-based per SDTMIG v3.4 Section 6.3.5 (Yes/No)</t>
+          <t>Section number in SDTMIG v3.4 where the domain is specified</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Measurement</t>
+          <t>Has_Test_Codes</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Whether the domain is a subject-level measurement domain (VS, EG, MK, CV) (Yes/No). EG included in flag despite deferred consumer status.</t>
+          <t>Whether the domain uses --TESTCD/--TEST variables (Yes/No)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>Specimen_Based</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Whether the domain is specimen-based per SDTMIG v3.4 Section 6.3.5 (Yes/No)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Whether the domain is a subject-level measurement domain (VS, EG, MK, CV) (Yes/No). EG included in flag despite deferred consumer status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Brief notes on domain status or version history</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr"/>
-      <c r="B27" s="2" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>KNOWN LIMITATIONS</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n"/>
-    </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Variable-level metadata (key variables, permissible variables) is not included.</t>
-        </is>
-      </c>
+      <c r="A29" s="2" t="inlineStr"/>
       <c r="B29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>That requires CDISC membership access to the SDTM v2.0 Excel files.</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="n"/>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>CODELIST_OVERRIDES COLUMNS</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>SDTM v3.0 is under review and may add or change domains.</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n"/>
+          <t>CT_Display_Name</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>The codelist display name from NCI EVS (after stripping " Test Code")</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>MO (Morphology) was decommissioned in v3.4 and is not listed.</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n"/>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Target SDTM domain abbreviation</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t>Override_Type</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Naming (label mismatch) or Subset (body-system sub-codelist)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Description of the mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>INSTRUMENT_DOMAIN_RULES COLUMNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Substring matched against codelist display name</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Target SDTM domain abbreviation</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Description and examples of instrument types in this category</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>KNOWN LIMITATIONS</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Variable-level metadata (key variables, permissible variables) is not included.</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>That requires CDISC membership access to the SDTM v2.0 Excel files.</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>SDTM v3.0 is under review and may add or change domains.</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>MO (Morphology) was decommissioned in v3.4 and is not listed.</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>SDTMIG section numbers are reconstructed from public sources — verify against the IG.</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -791,7 +917,7 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -825,7 +951,7 @@
           <t>Specimen_Based</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Measurement</t>
         </is>
@@ -3028,4 +3154,267 @@
   <autoFilter ref="A1:G57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>CT_Display_Name</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Override_Type</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>SDTM Microscopic Findings</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Naming</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>CT uses "SDTM Microscopic Findings", IG uses "Microscopic Findings"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Musculoskeletal System Finding</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>MK</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Naming</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>CT uses singular "Finding", IG uses "Musculoskeletal System Findings"</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Urinary System</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Naming</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>CT uses "Urinary System", IG uses "Urinary System Findings"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SDTM Death Diagnosis and Details</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>DD</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Naming</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>CT uses "SDTM Death Diagnosis and Details", IG uses "Death Details"</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Holter ECG</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Subset</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Body-system subset of ECG Test Results (HETESTCD is subset of EGTESTCD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Oncology Response Assessment</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Subset</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Body-system subset of Disease Response and Clin Classification</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Questionnaire</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>QS</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>PRO/ClinRO instruments (e.g. PHQ-9, GAD-7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Functional Test</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Performance-based instruments (e.g. 6MWT, TUG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Clinical Classification</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Clinician rating scales (e.g. NYHA, CHA2DS2-VASc)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>